<commit_message>
Update project resources and configurations
- Updated userconfig.ini to change Mold ID from 21-1966002 to 21-1061033.
- Modified mainwindow.cpp to update application version from v4.12.26 to v5.2.4.
- Adjusted resources.qrc to include additional document files and reorganized existing entries.
- Enhanced SQL query preparation in chonyakeep.cpp for exporting history records.
- Increased the number of columns written in the Excel export function in sumokeep.cpp from 12 to 17.
- Updated binary files qrc_resources.o and sumokeep.o.
- Updated Excel document chonya_keep3.xlsx.
</commit_message>
<xml_diff>
--- a/ducument/chonya_keep3.xlsx
+++ b/ducument/chonya_keep3.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -1068,7 +1068,7 @@
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="9" style="2" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="9" style="2" customWidth="1"/>
     <col min="2" max="2" width="15.0666666666667" style="2" customWidth="1"/>
     <col min="3" max="3" width="8.73333333333333" style="2" customWidth="1"/>
     <col min="4" max="4" width="19.6916666666667" style="2" customWidth="1"/>

</xml_diff>